<commit_message>
Added Rolf Hertz Lab Values
</commit_message>
<xml_diff>
--- a/scripts/modify_LIS_scripts/Laborwerte_zum_behalten_19_01_26.xlsx
+++ b/scripts/modify_LIS_scripts/Laborwerte_zum_behalten_19_01_26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniheidelbergde-my.sharepoint.com/personal/wa227_uni-heidelberg_de/Documents/IMI/HeiCuDigiMed/studiKIS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Workspace\Bahmni_Project\KIS-Projekt\scripts\modify_LIS_scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{DCF42DEF-39EE-4679-8D11-25A044442D68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E29A6561-7F6F-4167-B01E-7FA2E827B0A5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBC5CA11-27D9-40CA-9BBC-9672E6DCD549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="280">
   <si>
     <t>Name</t>
   </si>
@@ -858,6 +858,24 @@
   </si>
   <si>
     <t>Antithrombin III (AT-III)</t>
+  </si>
+  <si>
+    <t>GFR nach CKD-EPI</t>
+  </si>
+  <si>
+    <t>NT-pro-BNP</t>
+  </si>
+  <si>
+    <t>166017AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+  </si>
+  <si>
+    <t>N-terminal pro brain natriuretic peptide (NT-proBNP) measurement</t>
+  </si>
+  <si>
+    <t>Glomerular filtration rate, calculated</t>
+  </si>
+  <si>
+    <t>161133AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
   </si>
 </sst>
 </file>
@@ -1214,15 +1232,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C102"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.15234375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C104"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="67.3046875" customWidth="1"/>
-    <col min="2" max="2" width="44.15234375" customWidth="1"/>
-    <col min="3" max="3" width="56.84375" customWidth="1"/>
+    <col min="1" max="1" width="67.28515625" customWidth="1"/>
+    <col min="2" max="2" width="44.140625" customWidth="1"/>
+    <col min="3" max="3" width="56.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1233,7 +1251,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1244,7 +1262,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1255,7 +1273,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1266,7 +1284,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1277,7 +1295,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1288,7 +1306,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1299,7 +1317,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1310,7 +1328,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="3" t="s">
         <v>24</v>
@@ -1319,7 +1337,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -1330,7 +1348,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -1341,7 +1359,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -1352,7 +1370,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -1363,7 +1381,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -1374,7 +1392,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>41</v>
       </c>
@@ -1385,7 +1403,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>44</v>
       </c>
@@ -1396,7 +1414,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>47</v>
       </c>
@@ -1407,7 +1425,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>50</v>
       </c>
@@ -1418,7 +1436,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>53</v>
       </c>
@@ -1429,7 +1447,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>55</v>
       </c>
@@ -1440,7 +1458,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -1451,7 +1469,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>59</v>
       </c>
@@ -1462,7 +1480,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>62</v>
       </c>
@@ -1473,7 +1491,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>65</v>
       </c>
@@ -1484,7 +1502,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>68</v>
       </c>
@@ -1495,7 +1513,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>71</v>
       </c>
@@ -1506,7 +1524,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>74</v>
       </c>
@@ -1517,7 +1535,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>77</v>
       </c>
@@ -1528,7 +1546,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>80</v>
       </c>
@@ -1539,7 +1557,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>82</v>
       </c>
@@ -1550,7 +1568,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>85</v>
       </c>
@@ -1561,7 +1579,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>88</v>
       </c>
@@ -1572,7 +1590,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>91</v>
       </c>
@@ -1583,7 +1601,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>94</v>
       </c>
@@ -1594,7 +1612,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>97</v>
       </c>
@@ -1605,7 +1623,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>100</v>
       </c>
@@ -1616,7 +1634,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>103</v>
       </c>
@@ -1627,7 +1645,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>106</v>
       </c>
@@ -1638,7 +1656,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>109</v>
       </c>
@@ -1649,7 +1667,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>112</v>
       </c>
@@ -1660,7 +1678,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>115</v>
       </c>
@@ -1671,7 +1689,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>118</v>
       </c>
@@ -1682,7 +1700,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>121</v>
       </c>
@@ -1693,7 +1711,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="3" t="s">
         <v>124</v>
@@ -1702,7 +1720,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>126</v>
       </c>
@@ -1713,7 +1731,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>129</v>
       </c>
@@ -1724,7 +1742,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>132</v>
       </c>
@@ -1735,7 +1753,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="3" t="s">
         <v>135</v>
@@ -1744,7 +1762,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>137</v>
       </c>
@@ -1755,7 +1773,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>140</v>
       </c>
@@ -1766,7 +1784,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>143</v>
       </c>
@@ -1777,7 +1795,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>146</v>
       </c>
@@ -1788,7 +1806,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
       <c r="B53" s="3" t="s">
         <v>149</v>
@@ -1797,7 +1815,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>151</v>
       </c>
@@ -1808,7 +1826,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
       <c r="B55" s="3" t="s">
         <v>154</v>
@@ -1817,7 +1835,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>156</v>
       </c>
@@ -1828,7 +1846,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>159</v>
       </c>
@@ -1839,7 +1857,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>162</v>
       </c>
@@ -1850,7 +1868,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>165</v>
       </c>
@@ -1861,7 +1879,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>168</v>
       </c>
@@ -1872,7 +1890,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>171</v>
       </c>
@@ -1883,7 +1901,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>174</v>
       </c>
@@ -1894,7 +1912,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>177</v>
       </c>
@@ -1905,7 +1923,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>180</v>
       </c>
@@ -1916,7 +1934,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>183</v>
       </c>
@@ -1927,7 +1945,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>186</v>
       </c>
@@ -1938,7 +1956,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>189</v>
       </c>
@@ -1949,7 +1967,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>192</v>
       </c>
@@ -1960,7 +1978,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>195</v>
       </c>
@@ -1971,7 +1989,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>198</v>
       </c>
@@ -1982,7 +2000,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>201</v>
       </c>
@@ -1993,7 +2011,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>204</v>
       </c>
@@ -2004,7 +2022,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>207</v>
       </c>
@@ -2015,7 +2033,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="3"/>
       <c r="B74" s="3" t="s">
         <v>210</v>
@@ -2024,7 +2042,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="3"/>
       <c r="B75" s="3" t="s">
         <v>212</v>
@@ -2033,7 +2051,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>213</v>
       </c>
@@ -2044,7 +2062,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>216</v>
       </c>
@@ -2055,7 +2073,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="3"/>
       <c r="B78" s="3" t="s">
         <v>219</v>
@@ -2064,7 +2082,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>221</v>
       </c>
@@ -2075,7 +2093,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>224</v>
       </c>
@@ -2086,7 +2104,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="3"/>
       <c r="B81" s="3" t="s">
         <v>227</v>
@@ -2095,7 +2113,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="3"/>
       <c r="B82" s="3" t="s">
         <v>229</v>
@@ -2104,7 +2122,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>231</v>
       </c>
@@ -2115,7 +2133,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>234</v>
       </c>
@@ -2126,132 +2144,154 @@
         <v>236</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A87" s="2" t="s">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>278</v>
+      </c>
+      <c r="B85" t="s">
+        <v>274</v>
+      </c>
+      <c r="C85" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>277</v>
+      </c>
+      <c r="B86" t="s">
+        <v>275</v>
+      </c>
+      <c r="C86" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" s="2" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A88" t="s">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>238</v>
       </c>
-      <c r="B88" s="4" t="s">
+      <c r="B90" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="C88" t="s">
+      <c r="C90" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A89" t="s">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>240</v>
       </c>
-      <c r="B89" s="4" t="s">
+      <c r="B91" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="C89" t="s">
+      <c r="C91" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A90" t="s">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>242</v>
       </c>
-      <c r="B90" s="4" t="s">
+      <c r="B92" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="C90" t="s">
+      <c r="C92" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A91" t="s">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>244</v>
       </c>
-      <c r="B91" s="4" t="s">
+      <c r="B93" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="C91" t="s">
+      <c r="C93" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A92" t="s">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>246</v>
       </c>
-      <c r="B92" s="4" t="s">
+      <c r="B94" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="C92" t="s">
+      <c r="C94" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A93" t="s">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>248</v>
       </c>
-      <c r="B93" s="4" t="s">
+      <c r="B95" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="C93" t="s">
+      <c r="C95" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A94" t="s">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>250</v>
       </c>
-      <c r="B94" s="4" t="s">
+      <c r="B96" s="4" t="s">
         <v>265</v>
       </c>
-      <c r="C94" t="s">
+      <c r="C96" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A95" t="s">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>252</v>
       </c>
-      <c r="B95" s="4" t="s">
+      <c r="B97" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="C95" t="s">
+      <c r="C97" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="B96" s="4"/>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A97" s="2" t="s">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B98" s="4"/>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="B97" s="4"/>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A98" t="s">
+      <c r="B99" s="4"/>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>255</v>
       </c>
-      <c r="B98" s="4" t="s">
+      <c r="B100" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="C98" t="s">
+      <c r="C100" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A99" t="s">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>257</v>
       </c>
-      <c r="B99" s="4" t="s">
+      <c r="B101" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="C99" t="s">
+      <c r="C101" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A102" s="3" t="s">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" s="3" t="s">
         <v>259</v>
       </c>
     </row>

</xml_diff>